<commit_message>
Atualiza inventário com contagens precisas: 48 seringas azuis, 10 verdes, 2 packs pinça/tesoura, 130 gazes, 19 frascos
</commit_message>
<xml_diff>
--- a/Inventario_Material_Medico_FYTLOQ_Completo.xlsx
+++ b/Inventario_Material_Medico_FYTLOQ_Completo.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -553,11 +553,11 @@
       <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Seringas Azuis (individuais)</t>
+          <t>Seringas Azuis (cartelas)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
@@ -566,7 +566,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Seringas estéreis, vários tamanhos</t>
+          <t>4 cartelas com 12 seringas cada</t>
         </is>
       </c>
     </row>
@@ -574,11 +574,11 @@
       <c r="A7" s="5" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Seringas Verdes (individuais)</t>
+          <t>Seringas Verdes (cartela)</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
@@ -587,47 +587,47 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Seringas estéreis tamanho grande</t>
+          <t>1 cartela com 10 seringas</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Seringas Alaranjadas (pequenas)</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Seringas pequenas estéreis</t>
-        </is>
-      </c>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>LUVAS</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>LUVAS</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr"/>
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>DuPont Tyvek - Luvas Proteção</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>emb</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Embalagem completa XXL</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>DuPont Tyvek - Luvas Proteção</t>
+          <t>Luvas Nitrile Azuis</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
@@ -640,51 +640,51 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Embalagem completa XXL</t>
+          <t>Luvas de nitrilo estéreis</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Luvas Nitrile Azuis</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>caixa</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Luvas de nitrilo estéreis</t>
-        </is>
-      </c>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>BATAS/AVENTAIS</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>BATAS/AVENTAIS</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr"/>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr"/>
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Batas Cirúrgicas DocWorld Azuis</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Tamanho L, embalagem estéril</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr"/>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Batas Cirúrgicas DocWorld Azuis</t>
+          <t>Bata Tyvek</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
@@ -693,102 +693,92 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Tamanho L, embalagem estéril</t>
+          <t>Proteção descartável</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr"/>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Aventais Proteção Pessoal</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Embalagem completa</t>
-        </is>
-      </c>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>GAZES/COMPRESSAS</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>GAZES/COMPRESSAS</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr"/>
-      <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr"/>
+      <c r="A15" s="5" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Gazes/Compressas (packs)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Embalagens de gazes estéreis</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr"/>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Compressas Suprême - Pequenas</t>
+          <t>Gazes individuais embaladas</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>unid</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Gazes estéreis 5x5 cm</t>
+          <t>Gazes brancas embaladas</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr"/>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Compressas Suprême - Médias</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>pack</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Gazes estéreis 10x10 cm</t>
-        </is>
-      </c>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>FITAS ADESIVAS</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr"/>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr"/>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Compressas Suprême - Grandes</t>
+          <t>Tape Médico Branco</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>rolo</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Gazes estéreis 20x20 cm</t>
+          <t>Fita adesiva cirúrgica padrão</t>
         </is>
       </c>
     </row>
@@ -796,27 +786,27 @@
       <c r="A19" s="5" t="inlineStr"/>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Compressas verdes (em bandeja)</t>
+          <t>Tape Médico Cor Pele</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>bandeja</t>
+          <t>rolo</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Compressas estéreis verdes pré-corte</t>
+          <t>Fita adesiva discreta</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>PENSOS/CURATIVOS</t>
+          <t>SOLUÇÕES/FRASCOS</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr"/>
@@ -828,11 +818,11 @@
       <c r="A21" s="5" t="inlineStr"/>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Aluevyn - Pensos com almofada</t>
+          <t>Flacons redondos medicinais</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
@@ -841,7 +831,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Curativos com absorvente</t>
+          <t>Frascos com etiqueta</t>
         </is>
       </c>
     </row>
@@ -849,11 +839,11 @@
       <c r="A22" s="5" t="inlineStr"/>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>ElevasTrip - Kits curativos</t>
+          <t>Frascos/Garrafas adicionais</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -862,56 +852,46 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Sistemas de curativos estéreis</t>
+          <t>Soluções médicas variadas</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>DocWorld - Pensos variados</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>pack</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Diferentes tipos de curativos</t>
-        </is>
-      </c>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>TUBOS/IRRIGAÇÃO</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr"/>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Pensos Coloridos (laranja/rosa)</t>
+          <t>Tubo Transparente Enrolado</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>unid</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Curativos decorativos estéreis</t>
+          <t>Tubo de drenagem/irrigação</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>FITAS ADESIVAS</t>
+          <t>INSTRUMENTOS</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr"/>
@@ -923,7 +903,7 @@
       <c r="A26" s="5" t="inlineStr"/>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Tape Médico Branco</t>
+          <t>Packs com pinça/tesoura</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
@@ -931,283 +911,92 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>rolo</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Fita adesiva cirúrgica padrão</t>
+          <t>1 pinça + 1 tesoura por pack</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr"/>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Tape Médico Cor Pele</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>rolo</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Fita adesiva discreta</t>
-        </is>
-      </c>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>PROTEÇÃO CAPILAR</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr"/>
-      <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr"/>
+      <c r="A28" s="5" t="inlineStr"/>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Bonés/Coifas Médicos</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>unid</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Proteção capilar descartável</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Frasco Solução Transparente</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Solução salina/irrigação</t>
-        </is>
-      </c>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>DOCUMENTAÇÃO</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr"/>
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr"/>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Frascos Adicionais</t>
+          <t>Instruções/Manuais</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>unid</t>
+          <t>lote</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Soluções médicas variadas</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>TUBOS/IRRIGAÇÃO</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="4" t="inlineStr"/>
+          <t>Folhas de instruções variadas</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr"/>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Tubo Transparente Enrolado</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Tubo de drenagem/irrigação</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>INSTRUMENTOS</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Pinças/Tesouras Coloridas</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Rosa, azul, verde - uso único</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>PROTEÇÃO CAPILAR</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Bonés/Coifas Verdes</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>unid</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Proteção capilar descartável</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>DOCUMENTAÇÃO</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr"/>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Folhas Instruções Suprême</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>folha</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Instruções de produtos</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr"/>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Folhas Instruções DocWorld</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>folha</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Guias de utilização</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>3M PRODUTOS</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr"/>
-      <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="4" t="inlineStr"/>
-      <c r="E40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr"/>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Produtos 3M Variados</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>pack</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Curativos e proteção 3M</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>TOTAL DE ITENS</t>
         </is>
       </c>
-      <c r="C43" s="8">
+      <c r="C32" s="8">
         <f>SUM(C5:C50)</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="9" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>Inventário completo com contagens reais. Todos os itens estão em embalagem estéril e original. Pronto para uso clínico.</t>
         </is>
@@ -1216,9 +1005,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A45:E45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>